<commit_message>
hire history and other changes
</commit_message>
<xml_diff>
--- a/public/files/products_export.xlsx
+++ b/public/files/products_export.xlsx
@@ -309,7 +309,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -338,15 +338,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>177120</xdr:colOff>
+      <xdr:colOff>315000</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>142920</xdr:rowOff>
+      <xdr:rowOff>57240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>597240</xdr:colOff>
+      <xdr:colOff>734760</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>686520</xdr:rowOff>
+      <xdr:rowOff>600480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -359,8 +359,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="21464400">
-          <a:off x="977040" y="333360"/>
-          <a:ext cx="420120" cy="543600"/>
+          <a:off x="1115280" y="247320"/>
+          <a:ext cx="419760" cy="543240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -376,15 +376,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>84960</xdr:colOff>
+      <xdr:colOff>320760</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>96840</xdr:rowOff>
+      <xdr:rowOff>163800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>433800</xdr:colOff>
+      <xdr:colOff>669240</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>417240</xdr:rowOff>
+      <xdr:rowOff>483840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -397,8 +397,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="885240" y="2182680"/>
-          <a:ext cx="348840" cy="320400"/>
+          <a:off x="1121040" y="1093320"/>
+          <a:ext cx="348480" cy="320040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -414,15 +414,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>85320</xdr:colOff>
+      <xdr:colOff>242640</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>96840</xdr:rowOff>
+      <xdr:rowOff>230760</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>538920</xdr:colOff>
+      <xdr:colOff>695880</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>417240</xdr:rowOff>
+      <xdr:rowOff>550800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -435,8 +435,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="885600" y="2944800"/>
-          <a:ext cx="453600" cy="320400"/>
+          <a:off x="1042920" y="1922400"/>
+          <a:ext cx="453240" cy="320040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -451,16 +451,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>796680</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>1059840</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>311040</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>105120</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>335880</xdr:colOff>
+      <xdr:colOff>650160</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>318960</xdr:rowOff>
+      <xdr:rowOff>425160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -473,8 +473,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="796680" y="3907800"/>
-          <a:ext cx="339480" cy="320400"/>
+          <a:off x="1111320" y="2573280"/>
+          <a:ext cx="339120" cy="320040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -679,8 +679,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="11" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="26" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="11" style="1" width="15"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -759,21 +758,21 @@
       <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="0"/>
-      <c r="AA1" s="0"/>
-      <c r="AB1" s="0"/>
-      <c r="AC1" s="0"/>
-      <c r="AD1" s="0"/>
-      <c r="AE1" s="0"/>
-      <c r="AF1" s="0"/>
-      <c r="AG1" s="0"/>
-      <c r="AH1" s="0"/>
-      <c r="AI1" s="0"/>
-      <c r="AJ1" s="0"/>
-      <c r="AK1" s="0"/>
-      <c r="AL1" s="0"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="149.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="58.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -913,7 +912,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="83.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="61.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
         <v>42</v>
       </c>

</xml_diff>